<commit_message>
add regression framework results
</commit_message>
<xml_diff>
--- a/administrative/main.xlsx
+++ b/administrative/main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\GitHub\thesis\administrative\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6240DCC-66AD-408A-B7CA-CD84D1FF5B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F599DCF-7B95-4525-837C-84C6E14C0BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{4AC8BB16-67F5-4941-86E8-7E194268DB8A}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="302">
   <si>
     <t>Pandemics &amp; Diffussion Models</t>
   </si>
@@ -965,6 +965,12 @@
   </si>
   <si>
     <t>Ridge</t>
+  </si>
+  <si>
+    <t>Cases_t_1</t>
+  </si>
+  <si>
+    <t>Cases_t_4</t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1151,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1192,8 +1198,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3576,7 +3580,7 @@
       <c r="BN7" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="BO7" s="38">
+      <c r="BO7" s="14">
         <f>+_xlfn.XLOOKUP($BN7,$AX$7:$AX$10,$AZ$7:$AZ$10)</f>
         <v>22520.654823000001</v>
       </c>
@@ -3765,7 +3769,7 @@
       <c r="BN8" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="BO8" s="39">
+      <c r="BO8" s="17">
         <f t="shared" ref="BO8:BO10" si="9">+_xlfn.XLOOKUP($BN8,$AX$7:$AX$10,$AZ$7:$AZ$10)</f>
         <v>4703.6260300000004</v>
       </c>
@@ -3954,7 +3958,7 @@
       <c r="BN9" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="BO9" s="38">
+      <c r="BO9" s="14">
         <f t="shared" si="9"/>
         <v>2148.462321</v>
       </c>
@@ -4143,7 +4147,7 @@
       <c r="BN10" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="BO10" s="39">
+      <c r="BO10" s="17">
         <f t="shared" si="9"/>
         <v>53755.513460000002</v>
       </c>
@@ -7178,7 +7182,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93B5247-589C-44F9-8D52-5DE81A7C1480}">
-  <dimension ref="B1:CE26"/>
+  <dimension ref="B1:CE44"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
@@ -9284,6 +9288,9 @@
       <c r="CB19" s="13"/>
     </row>
     <row r="20" spans="34:80" x14ac:dyDescent="0.3">
+      <c r="AH20" s="1" t="s">
+        <v>250</v>
+      </c>
       <c r="BW20" s="19"/>
       <c r="BX20" s="19"/>
       <c r="BY20" s="19"/>
@@ -9328,25 +9335,25 @@
         <v>171</v>
       </c>
       <c r="AI22" s="14">
-        <v>7977465</v>
+        <v>8358205</v>
       </c>
       <c r="AJ22" s="14">
-        <v>6744284</v>
+        <v>6472772</v>
       </c>
       <c r="AK22" s="14">
-        <v>152178.4</v>
+        <v>247333.9</v>
       </c>
       <c r="AL22" s="14">
-        <v>179231.8</v>
+        <v>247360.9</v>
       </c>
       <c r="AM22" s="14">
-        <v>7386617</v>
+        <v>7119606</v>
       </c>
       <c r="AN22" s="14">
-        <v>908021.6</v>
+        <v>739199.5</v>
       </c>
       <c r="AO22" s="14">
-        <v>22672170</v>
+        <v>22672160</v>
       </c>
       <c r="BW22" s="13"/>
       <c r="BX22" s="13"/>
@@ -9360,22 +9367,22 @@
         <v>172</v>
       </c>
       <c r="AI23" s="14">
-        <v>3406131</v>
+        <v>3756126</v>
       </c>
       <c r="AJ23" s="14">
-        <v>1289262</v>
+        <v>1272250</v>
       </c>
       <c r="AK23" s="14">
-        <v>180850.8</v>
+        <v>141937.60000000001</v>
       </c>
       <c r="AL23" s="14">
-        <v>178724.6</v>
+        <v>141957.6</v>
       </c>
       <c r="AM23" s="14">
-        <v>1464898</v>
+        <v>1460144</v>
       </c>
       <c r="AN23" s="14">
-        <v>3359250</v>
+        <v>3376700</v>
       </c>
       <c r="AO23" s="14">
         <v>24316190</v>
@@ -9400,22 +9407,22 @@
         <v>175</v>
       </c>
       <c r="AI24" s="14">
-        <v>41910400</v>
+        <v>42386480</v>
       </c>
       <c r="AJ24" s="14">
-        <v>39159000</v>
+        <v>37853330</v>
       </c>
       <c r="AK24" s="14">
-        <v>2336516</v>
+        <v>2035471</v>
       </c>
       <c r="AL24" s="14">
-        <v>2336694</v>
+        <v>2035450</v>
       </c>
       <c r="AM24" s="14">
-        <v>40142750</v>
+        <v>40214680</v>
       </c>
       <c r="AN24" s="14">
-        <v>4643869</v>
+        <v>1304844</v>
       </c>
       <c r="AO24" s="14">
         <v>122159800</v>
@@ -9441,22 +9448,22 @@
         <v>176</v>
       </c>
       <c r="AI25" s="14">
-        <v>8240698</v>
+        <v>8256902</v>
       </c>
       <c r="AJ25" s="14">
-        <v>9073383</v>
+        <v>8702138</v>
       </c>
       <c r="AK25" s="14">
-        <v>357059.1</v>
+        <v>400986.7</v>
       </c>
       <c r="AL25" s="14">
-        <v>406927.1</v>
+        <v>401188.3</v>
       </c>
       <c r="AM25" s="14">
-        <v>8918761</v>
+        <v>8497244</v>
       </c>
       <c r="AN25" s="14">
-        <v>1458045</v>
+        <v>2367122</v>
       </c>
       <c r="AO25" s="14">
         <v>30861490</v>
@@ -9482,22 +9489,22 @@
         <v>179</v>
       </c>
       <c r="AI26" s="14">
-        <v>76685160</v>
+        <v>87020490</v>
       </c>
       <c r="AJ26" s="14">
-        <v>87278960</v>
+        <v>87979830</v>
       </c>
       <c r="AK26" s="14">
-        <v>3562568</v>
+        <v>3994550</v>
       </c>
       <c r="AL26" s="14">
-        <v>3704493</v>
+        <v>3993905</v>
       </c>
       <c r="AM26" s="14">
-        <v>103207900</v>
+        <v>99369740</v>
       </c>
       <c r="AN26" s="14">
-        <v>18045810</v>
+        <v>18872380</v>
       </c>
       <c r="AO26" s="14">
         <v>426086100</v>
@@ -9518,8 +9525,546 @@
       <c r="BT26" s="28"/>
       <c r="BU26" s="28"/>
     </row>
+    <row r="29" spans="34:80" x14ac:dyDescent="0.3">
+      <c r="AH29" s="29" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="30" spans="34:80" x14ac:dyDescent="0.3">
+      <c r="AH30" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI30" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="AJ30" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="AK30" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="AL30" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="AM30" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="AN30" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="AO30" s="9" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="31" spans="34:80" x14ac:dyDescent="0.3">
+      <c r="AH31" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="AI31" s="14">
+        <v>8448053</v>
+      </c>
+      <c r="AJ31" s="14">
+        <v>6780585</v>
+      </c>
+      <c r="AK31" s="14">
+        <v>65899.95</v>
+      </c>
+      <c r="AL31" s="14">
+        <v>59433.07</v>
+      </c>
+      <c r="AM31" s="14">
+        <v>7730858</v>
+      </c>
+      <c r="AN31" s="14">
+        <v>772883.5</v>
+      </c>
+      <c r="AO31" s="14">
+        <v>22698710</v>
+      </c>
+    </row>
+    <row r="32" spans="34:80" x14ac:dyDescent="0.3">
+      <c r="AH32" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="AI32" s="14">
+        <v>3641375</v>
+      </c>
+      <c r="AJ32" s="14">
+        <v>1288990</v>
+      </c>
+      <c r="AK32" s="14">
+        <v>98367.06</v>
+      </c>
+      <c r="AL32" s="14">
+        <v>147808.5</v>
+      </c>
+      <c r="AM32" s="14">
+        <v>1442136</v>
+      </c>
+      <c r="AN32" s="14">
+        <v>3279935</v>
+      </c>
+      <c r="AO32" s="14">
+        <v>23558110</v>
+      </c>
+    </row>
+    <row r="33" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH33" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="AI33" s="14">
+        <v>44264800</v>
+      </c>
+      <c r="AJ33" s="14">
+        <v>39037660</v>
+      </c>
+      <c r="AK33" s="14">
+        <v>396822.9</v>
+      </c>
+      <c r="AL33" s="14">
+        <v>410083.2</v>
+      </c>
+      <c r="AM33" s="14">
+        <v>40922950</v>
+      </c>
+      <c r="AN33" s="14">
+        <v>2976958</v>
+      </c>
+      <c r="AO33" s="14">
+        <v>123353700</v>
+      </c>
+    </row>
+    <row r="34" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH34" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI34" s="14">
+        <v>8295826</v>
+      </c>
+      <c r="AJ34" s="14">
+        <v>8770232</v>
+      </c>
+      <c r="AK34" s="14">
+        <v>236383.9</v>
+      </c>
+      <c r="AL34" s="14">
+        <v>268165.8</v>
+      </c>
+      <c r="AM34" s="14">
+        <v>8565617</v>
+      </c>
+      <c r="AN34" s="14">
+        <v>2513404</v>
+      </c>
+      <c r="AO34" s="14">
+        <v>31047740</v>
+      </c>
+    </row>
+    <row r="35" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH35" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI35" s="14">
+        <v>88022780</v>
+      </c>
+      <c r="AJ35" s="14">
+        <v>81075680</v>
+      </c>
+      <c r="AK35" s="14">
+        <v>1296517</v>
+      </c>
+      <c r="AL35" s="14">
+        <v>1329986</v>
+      </c>
+      <c r="AM35" s="14">
+        <v>99065760</v>
+      </c>
+      <c r="AN35" s="14">
+        <v>19143400</v>
+      </c>
+      <c r="AO35" s="14">
+        <v>427453400</v>
+      </c>
+    </row>
+    <row r="38" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH38" s="1" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="39" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH39" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI39" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="AJ39" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="AK39" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="AL39" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="AM39" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="AN39" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="AO39" s="9" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="40" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH40" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="AI40" s="14">
+        <v>8300763</v>
+      </c>
+      <c r="AJ40" s="14">
+        <v>7395443</v>
+      </c>
+      <c r="AK40" s="14">
+        <v>408375.8</v>
+      </c>
+      <c r="AL40" s="14">
+        <v>408305.3</v>
+      </c>
+      <c r="AM40" s="14">
+        <v>7755566</v>
+      </c>
+      <c r="AN40" s="14">
+        <v>1238832</v>
+      </c>
+      <c r="AO40" s="14">
+        <v>22730730</v>
+      </c>
+    </row>
+    <row r="41" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH41" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="AI41" s="14">
+        <v>3779986</v>
+      </c>
+      <c r="AJ41" s="14">
+        <v>1261350</v>
+      </c>
+      <c r="AK41" s="14">
+        <v>2078308</v>
+      </c>
+      <c r="AL41" s="14">
+        <v>2078353</v>
+      </c>
+      <c r="AM41" s="14">
+        <v>1379444</v>
+      </c>
+      <c r="AN41" s="14">
+        <v>3793630</v>
+      </c>
+      <c r="AO41" s="14">
+        <v>21256790</v>
+      </c>
+    </row>
+    <row r="42" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH42" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="AI42" s="14">
+        <v>43990100</v>
+      </c>
+      <c r="AJ42" s="14">
+        <v>39106190</v>
+      </c>
+      <c r="AK42" s="14">
+        <v>3578022</v>
+      </c>
+      <c r="AL42" s="14">
+        <v>3578005</v>
+      </c>
+      <c r="AM42" s="14">
+        <v>44898540</v>
+      </c>
+      <c r="AN42" s="14">
+        <v>5110701</v>
+      </c>
+      <c r="AO42" s="14">
+        <v>127592700</v>
+      </c>
+    </row>
+    <row r="43" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH43" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI43" s="14">
+        <v>8065792</v>
+      </c>
+      <c r="AJ43" s="14">
+        <v>8527451</v>
+      </c>
+      <c r="AK43" s="14">
+        <v>2342675</v>
+      </c>
+      <c r="AL43" s="14">
+        <v>2342966</v>
+      </c>
+      <c r="AM43" s="14">
+        <v>8968693</v>
+      </c>
+      <c r="AN43" s="14">
+        <v>3263058</v>
+      </c>
+      <c r="AO43" s="14">
+        <v>31673230</v>
+      </c>
+    </row>
+    <row r="44" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AH44" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI44" s="14">
+        <v>80946790</v>
+      </c>
+      <c r="AJ44" s="14">
+        <v>78253060</v>
+      </c>
+      <c r="AK44" s="14">
+        <v>16474180</v>
+      </c>
+      <c r="AL44" s="14">
+        <v>16476130</v>
+      </c>
+      <c r="AM44" s="14">
+        <v>91963430</v>
+      </c>
+      <c r="AN44" s="14">
+        <v>19756890</v>
+      </c>
+      <c r="AO44" s="14">
+        <v>433487500</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="AI7:AI16">
+    <cfRule type="colorScale" priority="59">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI22:AI26">
+    <cfRule type="colorScale" priority="36">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI22:AO22">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI23:AO23">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI24:AO24">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI25:AO25">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI26:AO26">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI7:AP7">
+    <cfRule type="colorScale" priority="51">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI8:AP8">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI9:AP9">
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI10:AP10">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI11:AP11">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI12:AP12">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI13:AP13">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI14:AP14">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI15:AP15">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI16:AP16">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ7:AJ16">
+    <cfRule type="colorScale" priority="58">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ22:AJ26">
     <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="min"/>
@@ -9531,8 +10076,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI7:AP7">
-    <cfRule type="colorScale" priority="27">
+  <conditionalFormatting sqref="AK7:AK16">
+    <cfRule type="colorScale" priority="57">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9543,8 +10088,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI8:AP8">
-    <cfRule type="colorScale" priority="26">
+  <conditionalFormatting sqref="AK22:AK26">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9555,8 +10100,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI9:AP9">
-    <cfRule type="colorScale" priority="25">
+  <conditionalFormatting sqref="AL7:AL16">
+    <cfRule type="colorScale" priority="56">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9567,7 +10112,175 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI10:AP10">
+  <conditionalFormatting sqref="AL22:AL26">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM7:AM16">
+    <cfRule type="colorScale" priority="55">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM22:AM26">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN7:AN16">
+    <cfRule type="colorScale" priority="54">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN22:AN26">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO7:AO16">
+    <cfRule type="colorScale" priority="53">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO22:AO26">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP7:AP16">
+    <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BC13:BE16 BG13:BI16 BK13:BM16 BO13:BQ16">
+    <cfRule type="colorScale" priority="74">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BS13:BU16">
+    <cfRule type="colorScale" priority="62">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BX7:CE7">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BX8:CE8">
+    <cfRule type="colorScale" priority="39">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BX9:CE9">
+    <cfRule type="colorScale" priority="38">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BX10:CE10">
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI31:AI35">
     <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
@@ -9579,7 +10292,79 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI11:AP11">
+  <conditionalFormatting sqref="AI31:AO31">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI32:AO32">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI33:AO33">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI34:AO34">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI35:AO35">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ31:AJ35">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK31:AK35">
     <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
@@ -9591,7 +10376,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI12:AP12">
+  <conditionalFormatting sqref="AL31:AL35">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
@@ -9603,7 +10388,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI13:AP13">
+  <conditionalFormatting sqref="AM31:AM35">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -9615,7 +10400,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI14:AP14">
+  <conditionalFormatting sqref="AN31:AN35">
     <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
@@ -9627,7 +10412,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI15:AP15">
+  <conditionalFormatting sqref="AO31:AO35">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
@@ -9639,175 +10424,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI16:AP16">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ7:AJ16">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK7:AK16">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL7:AL16">
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM7:AM16">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN7:AN16">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO7:AO16">
-    <cfRule type="colorScale" priority="29">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP7:AP16">
-    <cfRule type="colorScale" priority="28">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BC13:BE16 BG13:BI16 BK13:BM16 BO13:BQ16">
-    <cfRule type="colorScale" priority="50">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BS13:BU16">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX7:CE7">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX8:CE8">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX9:CE9">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX10:CE10">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI22:AI26">
+  <conditionalFormatting sqref="AI40:AI44">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -9819,7 +10436,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI22:AO22">
+  <conditionalFormatting sqref="AI40:AO40">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -9831,7 +10448,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI23:AO23">
+  <conditionalFormatting sqref="AI41:AO41">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -9843,7 +10460,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI24:AO24">
+  <conditionalFormatting sqref="AI42:AO42">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -9855,7 +10472,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI25:AO25">
+  <conditionalFormatting sqref="AI43:AO43">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -9867,7 +10484,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI26:AO26">
+  <conditionalFormatting sqref="AI44:AO44">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -9879,7 +10496,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ22:AJ26">
+  <conditionalFormatting sqref="AJ40:AJ44">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -9891,7 +10508,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK22:AK26">
+  <conditionalFormatting sqref="AK40:AK44">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -9903,7 +10520,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL22:AL26">
+  <conditionalFormatting sqref="AL40:AL44">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -9915,7 +10532,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM22:AM26">
+  <conditionalFormatting sqref="AM40:AM44">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -9927,7 +10544,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AN22:AN26">
+  <conditionalFormatting sqref="AN40:AN44">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -9939,7 +10556,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO22:AO26">
+  <conditionalFormatting sqref="AO40:AO44">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
add var model and results covid
</commit_message>
<xml_diff>
--- a/administrative/main.xlsx
+++ b/administrative/main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\GitHub\thesis\administrative\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F599DCF-7B95-4525-837C-84C6E14C0BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B842F594-9C25-43B9-B9E6-900E327DED9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{4AC8BB16-67F5-4941-86E8-7E194268DB8A}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="323">
   <si>
     <t>Pandemics &amp; Diffussion Models</t>
   </si>
@@ -971,6 +971,69 @@
   </si>
   <si>
     <t>Cases_t_4</t>
+  </si>
+  <si>
+    <t>const</t>
+  </si>
+  <si>
+    <t>L1.cases</t>
+  </si>
+  <si>
+    <t>L2.cases</t>
+  </si>
+  <si>
+    <t>L3.cases</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>L4.cases</t>
+  </si>
+  <si>
+    <t>L4.no2</t>
+  </si>
+  <si>
+    <t>L5.cases</t>
+  </si>
+  <si>
+    <t>VAR cases log</t>
+  </si>
+  <si>
+    <t>L1.o3</t>
+  </si>
+  <si>
+    <t>L2.Mean_distance_avg_14day_movavg</t>
+  </si>
+  <si>
+    <t>L3.no2</t>
+  </si>
+  <si>
+    <t>L4.o3</t>
+  </si>
+  <si>
+    <t>L5.o3</t>
+  </si>
+  <si>
+    <t>L3.o3</t>
+  </si>
+  <si>
+    <t>L4.Mean_distance_avg_14day_movavg</t>
+  </si>
+  <si>
+    <t>L5.Mean_distance_avg_14day_movavg</t>
+  </si>
+  <si>
+    <t>L1.pm25</t>
+  </si>
+  <si>
+    <t>L4.pm25</t>
+  </si>
+  <si>
+    <t>L5.pm25</t>
+  </si>
+  <si>
+    <t>VAR</t>
   </si>
 </sst>
 </file>
@@ -7182,7 +7245,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93B5247-589C-44F9-8D52-5DE81A7C1480}">
-  <dimension ref="B1:CE44"/>
+  <dimension ref="B1:CE60"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
@@ -9555,6 +9618,9 @@
       <c r="AO30" s="9" t="s">
         <v>233</v>
       </c>
+      <c r="AP30" s="9" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="31" spans="34:80" x14ac:dyDescent="0.3">
       <c r="AH31" s="1" t="s">
@@ -9581,6 +9647,9 @@
       <c r="AO31" s="14">
         <v>22698710</v>
       </c>
+      <c r="AP31" s="14">
+        <v>4344672</v>
+      </c>
     </row>
     <row r="32" spans="34:80" x14ac:dyDescent="0.3">
       <c r="AH32" s="6" t="s">
@@ -9607,8 +9676,11 @@
       <c r="AO32" s="14">
         <v>23558110</v>
       </c>
-    </row>
-    <row r="33" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP32" s="14">
+        <v>2015265</v>
+      </c>
+    </row>
+    <row r="33" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH33" s="1" t="s">
         <v>175</v>
       </c>
@@ -9633,8 +9705,11 @@
       <c r="AO33" s="14">
         <v>123353700</v>
       </c>
-    </row>
-    <row r="34" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP33" s="14">
+        <v>152331600</v>
+      </c>
+    </row>
+    <row r="34" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH34" s="6" t="s">
         <v>176</v>
       </c>
@@ -9659,8 +9734,11 @@
       <c r="AO34" s="14">
         <v>31047740</v>
       </c>
-    </row>
-    <row r="35" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP34" s="14">
+        <v>3783188</v>
+      </c>
+    </row>
+    <row r="35" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH35" s="1" t="s">
         <v>179</v>
       </c>
@@ -9685,13 +9763,16 @@
       <c r="AO35" s="14">
         <v>427453400</v>
       </c>
-    </row>
-    <row r="38" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP35" s="14">
+        <v>228807800</v>
+      </c>
+    </row>
+    <row r="38" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH38" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="39" spans="34:41" x14ac:dyDescent="0.3">
+    <row r="39" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH39" s="9" t="s">
         <v>165</v>
       </c>
@@ -9717,7 +9798,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="40" spans="34:41" x14ac:dyDescent="0.3">
+    <row r="40" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH40" s="1" t="s">
         <v>171</v>
       </c>
@@ -9742,8 +9823,9 @@
       <c r="AO40" s="14">
         <v>22730730</v>
       </c>
-    </row>
-    <row r="41" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP40" s="14"/>
+    </row>
+    <row r="41" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH41" s="6" t="s">
         <v>172</v>
       </c>
@@ -9768,8 +9850,9 @@
       <c r="AO41" s="14">
         <v>21256790</v>
       </c>
-    </row>
-    <row r="42" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP41" s="14"/>
+    </row>
+    <row r="42" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH42" s="1" t="s">
         <v>175</v>
       </c>
@@ -9794,8 +9877,9 @@
       <c r="AO42" s="14">
         <v>127592700</v>
       </c>
-    </row>
-    <row r="43" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP42" s="14"/>
+    </row>
+    <row r="43" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH43" s="6" t="s">
         <v>176</v>
       </c>
@@ -9820,8 +9904,9 @@
       <c r="AO43" s="14">
         <v>31673230</v>
       </c>
-    </row>
-    <row r="44" spans="34:41" x14ac:dyDescent="0.3">
+      <c r="AP43" s="14"/>
+    </row>
+    <row r="44" spans="34:42" x14ac:dyDescent="0.3">
       <c r="AH44" s="1" t="s">
         <v>179</v>
       </c>
@@ -9846,9 +9931,526 @@
       <c r="AO44" s="14">
         <v>433487500</v>
       </c>
+      <c r="AP44" s="14"/>
+    </row>
+    <row r="49" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH49" s="1" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="50" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH50" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="AI50" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ50" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="AK50" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="AL50" s="9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="51" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH51" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="AI51" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="AJ51" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="AK51" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="AL51" s="1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="52" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH52" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="AI52" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="AJ52" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="AK52" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="AL52" s="6" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="53" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH53" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="AI53" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="AJ53" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="AK53" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL53" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="54" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH54" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="AI54" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="AJ54" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="AK54" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL54" s="6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="55" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH55" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="AI55" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="AJ55" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="AK55" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL55" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="56" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH56" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="AI56" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="AJ56" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="AK56" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL56" s="6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="57" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH57" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="AI57" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="AJ57" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AK57" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL57" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="58" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH58" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="AI58" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="AJ58" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AK58" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL58" s="6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="59" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH59" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AI59" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="AJ59" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AK59" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL59" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="60" spans="34:38" x14ac:dyDescent="0.3">
+      <c r="AH60" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AI60" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="AJ60" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AK60" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="AL60" s="6" t="s">
+        <v>306</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="AI7:AI16">
+    <cfRule type="colorScale" priority="76">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI22:AI26">
+    <cfRule type="colorScale" priority="53">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI31:AI35">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI40:AI44">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI22:AO22">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI23:AO23">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI24:AO24">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI25:AO25">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI26:AO26">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI31:AO31">
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI32:AO32">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI33:AO33">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI34:AO34">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI35:AO35">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI40:AP40">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI41:AP41">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI42:AP42">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI43:AP43">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI44:AP44">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI7:AP7">
+    <cfRule type="colorScale" priority="68">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI8:AP8">
+    <cfRule type="colorScale" priority="67">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI9:AP9">
+    <cfRule type="colorScale" priority="66">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI10:AP10">
+    <cfRule type="colorScale" priority="65">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI11:AP11">
+    <cfRule type="colorScale" priority="63">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI12:AP12">
+    <cfRule type="colorScale" priority="62">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI13:AP13">
+    <cfRule type="colorScale" priority="61">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI14:AP14">
+    <cfRule type="colorScale" priority="60">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI15:AP15">
     <cfRule type="colorScale" priority="59">
       <colorScale>
         <cfvo type="min"/>
@@ -9860,7 +10462,235 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI22:AI26">
+  <conditionalFormatting sqref="AI16:AP16">
+    <cfRule type="colorScale" priority="58">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ7:AJ16">
+    <cfRule type="colorScale" priority="75">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ22:AJ26">
+    <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ31:AJ35">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ40:AJ44">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK7:AK16">
+    <cfRule type="colorScale" priority="74">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK22:AK26">
+    <cfRule type="colorScale" priority="51">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK31:AK35">
+    <cfRule type="colorScale" priority="39">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK40:AK44">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL7:AL16">
+    <cfRule type="colorScale" priority="73">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL22:AL26">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL31:AL35">
+    <cfRule type="colorScale" priority="38">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL40:AL44">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM7:AM16">
+    <cfRule type="colorScale" priority="72">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM22:AM26">
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM31:AM35">
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM40:AM44">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN7:AN16">
+    <cfRule type="colorScale" priority="71">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN22:AN26">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN31:AN35">
     <cfRule type="colorScale" priority="36">
       <colorScale>
         <cfvo type="min"/>
@@ -9872,8 +10702,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI22:AO22">
-    <cfRule type="colorScale" priority="29">
+  <conditionalFormatting sqref="AN40:AN44">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9884,8 +10714,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI23:AO23">
-    <cfRule type="colorScale" priority="28">
+  <conditionalFormatting sqref="AO7:AO16">
+    <cfRule type="colorScale" priority="70">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9896,8 +10726,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI24:AO24">
-    <cfRule type="colorScale" priority="27">
+  <conditionalFormatting sqref="AO22:AO26">
+    <cfRule type="colorScale" priority="47">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9908,163 +10738,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI25:AO25">
-    <cfRule type="colorScale" priority="26">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI26:AO26">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI7:AP7">
-    <cfRule type="colorScale" priority="51">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI8:AP8">
-    <cfRule type="colorScale" priority="50">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI9:AP9">
-    <cfRule type="colorScale" priority="49">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI10:AP10">
-    <cfRule type="colorScale" priority="48">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI11:AP11">
-    <cfRule type="colorScale" priority="46">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI12:AP12">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI13:AP13">
-    <cfRule type="colorScale" priority="44">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI14:AP14">
-    <cfRule type="colorScale" priority="43">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI15:AP15">
-    <cfRule type="colorScale" priority="42">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI16:AP16">
-    <cfRule type="colorScale" priority="41">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ7:AJ16">
-    <cfRule type="colorScale" priority="58">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ22:AJ26">
+  <conditionalFormatting sqref="AO31:AO35">
     <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="min"/>
@@ -10076,7 +10750,55 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK7:AK16">
+  <conditionalFormatting sqref="AO40:AO44">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP7:AP16">
+    <cfRule type="colorScale" priority="69">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BC13:BE16 BG13:BI16 BK13:BM16 BO13:BQ16">
+    <cfRule type="colorScale" priority="91">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BS13:BU16">
+    <cfRule type="colorScale" priority="79">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BX7:CE7">
     <cfRule type="colorScale" priority="57">
       <colorScale>
         <cfvo type="min"/>
@@ -10088,19 +10810,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK22:AK26">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL7:AL16">
+  <conditionalFormatting sqref="BX8:CE8">
     <cfRule type="colorScale" priority="56">
       <colorScale>
         <cfvo type="min"/>
@@ -10112,19 +10822,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL22:AL26">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM7:AM16">
+  <conditionalFormatting sqref="BX9:CE9">
     <cfRule type="colorScale" priority="55">
       <colorScale>
         <cfvo type="min"/>
@@ -10136,19 +10834,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM22:AM26">
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN7:AN16">
+  <conditionalFormatting sqref="BX10:CE10">
     <cfRule type="colorScale" priority="54">
       <colorScale>
         <cfvo type="min"/>
@@ -10160,139 +10846,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AN22:AN26">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO7:AO16">
-    <cfRule type="colorScale" priority="53">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO22:AO26">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP7:AP16">
-    <cfRule type="colorScale" priority="52">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BC13:BE16 BG13:BI16 BK13:BM16 BO13:BQ16">
-    <cfRule type="colorScale" priority="74">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BS13:BU16">
-    <cfRule type="colorScale" priority="62">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX7:CE7">
-    <cfRule type="colorScale" priority="40">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX8:CE8">
-    <cfRule type="colorScale" priority="39">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX9:CE9">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BX10:CE10">
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI31:AI35">
-    <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI31:AO31">
+  <conditionalFormatting sqref="AP40:AP44">
     <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
@@ -10304,8 +10858,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI32:AO32">
-    <cfRule type="colorScale" priority="16">
+  <conditionalFormatting sqref="AP31">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10316,8 +10870,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI33:AO33">
-    <cfRule type="colorScale" priority="15">
+  <conditionalFormatting sqref="AP32">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10328,8 +10882,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI34:AO34">
-    <cfRule type="colorScale" priority="14">
+  <conditionalFormatting sqref="AP33">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10340,8 +10894,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI35:AO35">
-    <cfRule type="colorScale" priority="13">
+  <conditionalFormatting sqref="AP34">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10352,8 +10906,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ31:AJ35">
-    <cfRule type="colorScale" priority="23">
+  <conditionalFormatting sqref="AP35">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10364,8 +10918,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK31:AK35">
-    <cfRule type="colorScale" priority="22">
+  <conditionalFormatting sqref="AP31:AP35">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10376,67 +10930,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL31:AL35">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM31:AM35">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN31:AN35">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO31:AO35">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI40:AI44">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI40:AO40">
+  <conditionalFormatting sqref="AI31:AP31">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -10448,7 +10942,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI41:AO41">
+  <conditionalFormatting sqref="AI32:AP32">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -10460,7 +10954,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI42:AO42">
+  <conditionalFormatting sqref="AI33:AP33">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -10472,7 +10966,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI43:AO43">
+  <conditionalFormatting sqref="AI34:AP34">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -10484,80 +10978,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI44:AO44">
+  <conditionalFormatting sqref="AI35:AP35">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ40:AJ44">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK40:AK44">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL40:AL44">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM40:AM44">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN40:AN44">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO40:AO44">
-    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
add google trends and meteo colombia
</commit_message>
<xml_diff>
--- a/administrative/main.xlsx
+++ b/administrative/main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\GitHub\thesis\administrative\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22D20B1-DF2F-4E22-9997-41AC0C1ACD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD79D47-8CD5-4D63-8AAC-D8024168CC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{4AC8BB16-67F5-4941-86E8-7E194268DB8A}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="327">
   <si>
     <t>Pandemics &amp; Diffussion Models</t>
   </si>
@@ -1040,6 +1040,12 @@
   </si>
   <si>
     <t>meteo colombia</t>
+  </si>
+  <si>
+    <t>https://trends.google.it/trends/explore?date=2020-01-01%202023-12-31&amp;geo=UY&amp;q=%2Fm%2F05t4q,%2Fm%2F0hpnr,%2Fm%2F01rfps,%2Fm%2F01b_06&amp;hl=en-GB</t>
+  </si>
+  <si>
+    <t>query google trends</t>
   </si>
 </sst>
 </file>
@@ -2147,7 +2153,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA430712-2AF2-46BC-B2A9-A9F8B8AAD612}">
-  <dimension ref="B1:E24"/>
+  <dimension ref="B1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
@@ -2334,6 +2340,14 @@
       </c>
       <c r="C24" s="1" t="s">
         <v>324</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B25" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -2358,6 +2372,7 @@
     <hyperlink ref="B22" r:id="rId18" xr:uid="{9A099B35-5ED8-4261-8DF9-3E66B98A53E9}"/>
     <hyperlink ref="B23" r:id="rId19" xr:uid="{147E40C6-D2E1-46D8-854B-3827BE9D5F5D}"/>
     <hyperlink ref="B24" r:id="rId20" xr:uid="{072E2C55-83F5-4678-A782-C260562B8B6B}"/>
+    <hyperlink ref="B25" r:id="rId21" xr:uid="{0B637547-4E97-4EC3-B314-56A41CE2A5A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add air pollution to epidemics
</commit_message>
<xml_diff>
--- a/administrative/main.xlsx
+++ b/administrative/main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\GitHub\thesis\administrative\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95322EF9-6CD9-4F00-A53B-602DC4A4A41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAC58CD-0470-4196-97D5-0434328969E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{4AC8BB16-67F5-4941-86E8-7E194268DB8A}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="354">
   <si>
     <t>Pandemics &amp; Diffussion Models</t>
   </si>
@@ -1090,15 +1090,9 @@
     <t>L3.chik_cumulative</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>L3.pres</t>
   </si>
   <si>
-    <t>L4.chik_cumulative</t>
-  </si>
-  <si>
     <t>L5.tavg</t>
   </si>
   <si>
@@ -1111,16 +1105,28 @@
     <t>L3.zika_cumulative</t>
   </si>
   <si>
-    <t>L3.tavg</t>
-  </si>
-  <si>
     <t>L4.zika_cumulative</t>
   </si>
   <si>
-    <t>L4.tavg</t>
-  </si>
-  <si>
     <t>t+1</t>
+  </si>
+  <si>
+    <t>L1.pm10</t>
+  </si>
+  <si>
+    <t>L1.pres</t>
+  </si>
+  <si>
+    <t>L3.google_hospital</t>
+  </si>
+  <si>
+    <t>L3.pm10</t>
+  </si>
+  <si>
+    <t>L5.humidity</t>
+  </si>
+  <si>
+    <t>L3.so2</t>
   </si>
 </sst>
 </file>
@@ -9177,7 +9183,7 @@
       <c r="BT14" s="14"/>
       <c r="BU14" s="14"/>
       <c r="BW14" s="1" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
     </row>
     <row r="15" spans="2:83" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -9468,25 +9474,25 @@
         <v>331</v>
       </c>
       <c r="BX16" s="14">
-        <v>7.3023619999999996</v>
+        <v>6.5000390000000001</v>
       </c>
       <c r="BY16" s="14">
-        <v>23.153338999999999</v>
+        <v>23.705583000000001</v>
       </c>
       <c r="BZ16" s="14">
-        <v>1.312649</v>
+        <v>1.312819</v>
       </c>
       <c r="CA16" s="14">
-        <v>1.6906680000000001</v>
+        <v>1.3858550000000001</v>
       </c>
       <c r="CB16" s="14">
-        <v>24.156554</v>
+        <v>24.441410999999999</v>
       </c>
       <c r="CC16" s="14">
-        <v>9.6223559999999999</v>
+        <v>9.3939389999999996</v>
       </c>
       <c r="CD16" s="14">
-        <v>107.470157</v>
+        <v>109.669701</v>
       </c>
       <c r="CE16" s="14">
         <v>31.725518000000001</v>
@@ -9497,28 +9503,28 @@
         <v>195</v>
       </c>
       <c r="BX17" s="17">
-        <v>27784.75676</v>
+        <v>28631.619245999998</v>
       </c>
       <c r="BY17" s="17">
-        <v>45692.435870000001</v>
+        <v>45811.162887999999</v>
       </c>
       <c r="BZ17" s="17">
-        <v>831.05332099999998</v>
+        <v>937.95254799999998</v>
       </c>
       <c r="CA17" s="17">
-        <v>349.12991</v>
+        <v>450.39849199999998</v>
       </c>
       <c r="CB17" s="17">
-        <v>47565.684982999999</v>
+        <v>47791.344292000002</v>
       </c>
       <c r="CC17" s="17">
-        <v>13343.920405000001</v>
+        <v>14177.064490999999</v>
       </c>
       <c r="CD17" s="17">
-        <v>121114.350896</v>
+        <v>121112.837029</v>
       </c>
       <c r="CE17" s="17">
-        <v>6894.8666080000003</v>
+        <v>5855.042743</v>
       </c>
     </row>
     <row r="18" spans="34:83" x14ac:dyDescent="0.3">
@@ -9526,28 +9532,28 @@
         <v>332</v>
       </c>
       <c r="BX18" s="14">
-        <v>6912.7279230000004</v>
+        <v>7253.7510709999997</v>
       </c>
       <c r="BY18" s="14">
-        <v>16731.626419</v>
+        <v>16866.313760000001</v>
       </c>
       <c r="BZ18" s="14">
-        <v>1236.609516</v>
+        <v>2231.3267719999999</v>
       </c>
       <c r="CA18" s="14">
-        <v>66.889324000000002</v>
+        <v>57.783405999999999</v>
       </c>
       <c r="CB18" s="14">
-        <v>17334.479093000002</v>
+        <v>17332.664193000001</v>
       </c>
       <c r="CC18" s="14">
-        <v>657.88363900000002</v>
+        <v>928.31180199999994</v>
       </c>
       <c r="CD18" s="14">
-        <v>48215.132081999996</v>
+        <v>48213.643342000003</v>
       </c>
       <c r="CE18" s="14">
-        <v>8147.0878750000002</v>
+        <v>8510.9496409999992</v>
       </c>
     </row>
     <row r="19" spans="34:83" x14ac:dyDescent="0.3">
@@ -9555,28 +9561,28 @@
         <v>196</v>
       </c>
       <c r="BX19" s="17">
-        <v>12.758763999999999</v>
+        <v>11.312836000000001</v>
       </c>
       <c r="BY19" s="17">
-        <v>11.847369</v>
+        <v>11.884532</v>
       </c>
       <c r="BZ19" s="17">
-        <v>1.5559229999999999</v>
+        <v>1.5555490000000001</v>
       </c>
       <c r="CA19" s="17">
-        <v>1.591691</v>
+        <v>1.3179190000000001</v>
       </c>
       <c r="CB19" s="17">
-        <v>12.320406999999999</v>
+        <v>12.5166</v>
       </c>
       <c r="CC19" s="17">
-        <v>8.3875679999999999</v>
+        <v>9.2154480000000003</v>
       </c>
       <c r="CD19" s="17">
-        <v>67.611076999999995</v>
+        <v>70.252651999999998</v>
       </c>
       <c r="CE19" s="17">
-        <v>25.013144</v>
+        <v>16.767234999999999</v>
       </c>
     </row>
     <row r="20" spans="34:83" x14ac:dyDescent="0.3">
@@ -9837,7 +9843,7 @@
         <v>302</v>
       </c>
       <c r="BY27" s="1" t="s">
-        <v>333</v>
+        <v>302</v>
       </c>
       <c r="BZ27" s="1" t="s">
         <v>302</v>
@@ -9851,7 +9857,7 @@
         <v>334</v>
       </c>
       <c r="BY28" s="6" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="BZ28" s="6" t="s">
         <v>336</v>
@@ -9868,13 +9874,13 @@
         <v>338</v>
       </c>
       <c r="BY29" s="1" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="BZ29" s="1" t="s">
         <v>340</v>
       </c>
       <c r="CA29" s="1" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
     </row>
     <row r="30" spans="34:83" x14ac:dyDescent="0.3">
@@ -9906,16 +9912,16 @@
         <v>315</v>
       </c>
       <c r="BX30" s="6" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="BY30" s="6" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="BZ30" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="CA30" s="6" t="s">
-        <v>341</v>
+        <v>312</v>
       </c>
     </row>
     <row r="31" spans="34:83" x14ac:dyDescent="0.3">
@@ -9947,16 +9953,13 @@
         <v>7268706</v>
       </c>
       <c r="BX31" s="1" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="BY31" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="BZ31" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="CA31" s="1" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
     </row>
     <row r="32" spans="34:83" x14ac:dyDescent="0.3">
@@ -9988,16 +9991,14 @@
         <v>1387276</v>
       </c>
       <c r="BX32" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="BY32" s="6" t="s">
-        <v>347</v>
-      </c>
-      <c r="BZ32" s="6" t="s">
-        <v>341</v>
-      </c>
+        <v>312</v>
+      </c>
+      <c r="BZ32" s="6"/>
       <c r="CA32" s="6" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
     </row>
     <row r="33" spans="34:79" x14ac:dyDescent="0.3">
@@ -10029,16 +10030,13 @@
         <v>86397360</v>
       </c>
       <c r="BX33" s="1" t="s">
-        <v>341</v>
+        <v>352</v>
       </c>
       <c r="BY33" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="BZ33" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="CA33" s="1" t="s">
-        <v>341</v>
+        <v>309</v>
       </c>
     </row>
     <row r="34" spans="34:79" x14ac:dyDescent="0.3">
@@ -10069,18 +10067,12 @@
       <c r="AP34" s="14">
         <v>6536393</v>
       </c>
-      <c r="BX34" s="6" t="s">
-        <v>341</v>
-      </c>
+      <c r="BX34" s="6"/>
       <c r="BY34" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="BZ34" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="CA34" s="6" t="s">
-        <v>341</v>
-      </c>
+        <v>343</v>
+      </c>
+      <c r="BZ34" s="6"/>
+      <c r="CA34" s="6"/>
     </row>
     <row r="35" spans="34:79" x14ac:dyDescent="0.3">
       <c r="AH35" s="1" t="s">
@@ -10110,17 +10102,21 @@
       <c r="AP35" s="14">
         <v>259778200</v>
       </c>
-      <c r="BX35" s="1" t="s">
-        <v>341</v>
-      </c>
       <c r="BY35" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="BZ35" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="CA35" s="1" t="s">
-        <v>341</v>
+        <v>345</v>
+      </c>
+    </row>
+    <row r="36" spans="34:79" x14ac:dyDescent="0.3">
+      <c r="BX36" s="6"/>
+      <c r="BY36" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="BZ36" s="6"/>
+      <c r="CA36" s="6"/>
+    </row>
+    <row r="37" spans="34:79" x14ac:dyDescent="0.3">
+      <c r="BY37" s="1" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="38" spans="34:79" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fix ggm + arima
make r script for ggm + arima, simpler and more understandable
</commit_message>
<xml_diff>
--- a/administrative/main.xlsx
+++ b/administrative/main.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Documents\GitHub\thesis\administrative\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51007C25-6365-4EF8-B51A-773694D017B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4CE30C-C5DC-4F46-84AE-9BE0C422B0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{4AC8BB16-67F5-4941-86E8-7E194268DB8A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4AC8BB16-67F5-4941-86E8-7E194268DB8A}"/>
   </bookViews>
   <sheets>
     <sheet name="literature review" sheetId="1" r:id="rId1"/>
@@ -2108,6 +2108,9 @@
       <c r="E24" s="4" t="s">
         <v>208</v>
       </c>
+      <c r="F24" s="1" t="s">
+        <v>226</v>
+      </c>
       <c r="G24" s="39" t="s">
         <v>356</v>
       </c>
@@ -2124,9 +2127,6 @@
       </c>
       <c r="E25" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>226</v>
       </c>
       <c r="G25" s="39" t="s">
         <v>356</v>

</xml_diff>